<commit_message>
limpieza de archivos sensibles
</commit_message>
<xml_diff>
--- a/CHARMS BEADS DISNEY.xlsx
+++ b/CHARMS BEADS DISNEY.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\CATALOGO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A88BC1A-FA65-4A0A-823A-21A7A0959CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22438471-0991-476D-B68F-6C258CF1FE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0A3D0F50-D46A-4AA3-8C9D-74D0C1C259E3}"/>
   </bookViews>
@@ -12466,22 +12466,22 @@
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="8">
-        <v>3.42</v>
+        <v>3.16</v>
       </c>
       <c r="D6" s="9">
         <f t="shared" si="0"/>
-        <v>30.36</v>
+        <v>28.28</v>
       </c>
       <c r="E6" s="9">
         <f t="shared" si="1"/>
-        <v>60.72</v>
+        <v>56.56</v>
       </c>
       <c r="F6" s="9">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G6" s="9">
         <f t="shared" si="2"/>
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>

</xml_diff>